<commit_message>
Sesuaikan masterplan warkop untuk modal Rp 50 juta
Strategi naik kelas bertahap: kios kecil, kopi kekinian dari cold brew
dan moka pot, owner ikut operasional, upgrade espresso dari laba.
Model keuangan Excel diperbarui (BEP ±41 transaksi/hari).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjJU715WJBpBotxgoH1Pwh
</commit_message>
<xml_diff>
--- a/warkop/Model-Keuangan-Warkop.xlsx
+++ b/warkop/Model-Keuangan-Warkop.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>19000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="4">
@@ -540,21 +540,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sewa (amortisasi Rp24jt/tahun)</t>
+          <t>Sewa (Rp1,2jt/bulan)</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>2000000</v>
+        <v>1200000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Gaji 4 crew (2 per shift)</t>
+          <t>Gaji 2 crew</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>11200000</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="14">
@@ -564,17 +564,17 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>1800000</v>
+        <v>800000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Listrik (4.400 VA)</t>
+          <t>Listrik (2.200 VA)</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>2500000</v>
+        <v>1000000</v>
       </c>
     </row>
     <row r="16">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>1600000</v>
+        <v>1000000</v>
       </c>
     </row>
     <row r="17">
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>900000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="18">
@@ -604,17 +604,17 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>1500000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Langganan POS &amp; aplikasi</t>
+          <t>POS &amp; aplikasi (versi gratis)</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>300000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>700000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="21">
@@ -634,17 +634,17 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>800000</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Penyusutan alat, furniture &amp; sistem (± Rp52jt / 48 bln)</t>
+          <t>Penyusutan alat (± Rp20,4jt / 48 bln)</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>1200000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="23">
@@ -664,6 +664,14 @@
           <t>TARGET TRANSAKSI PER HARI (ramp-up)</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Bulan sewa dibayar di muka:</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -672,7 +680,7 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27">
@@ -682,7 +690,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
@@ -692,7 +700,7 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>95</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29">
@@ -702,7 +710,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30">
@@ -712,7 +720,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>115</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31">
@@ -722,7 +730,7 @@
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32">
@@ -732,7 +740,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>125</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33">
@@ -742,7 +750,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>130</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34">
@@ -752,7 +760,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>130</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35">
@@ -762,7 +770,7 @@
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>135</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36">
@@ -772,7 +780,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>135</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37">
@@ -782,7 +790,7 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>140</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -796,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -849,14 +857,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sewa kios/ruko 4x10 m, 1 tahun di muka</t>
+          <t>Sewa kios 3x8 m + teras, 6 bulan di muka (Rp1,2jt/bln)</t>
         </is>
       </c>
       <c r="C2" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>24000000</v>
+        <v>1200000</v>
       </c>
       <c r="E2" s="9">
         <f>C2*D2</f>
@@ -868,7 +876,7 @@
         </is>
       </c>
       <c r="H2" s="9">
-        <f>SUMIF($A$2:$A$44,G2,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G2,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -880,14 +888,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cat, mural &amp; finishing dinding</t>
+          <t>Cat &amp; mural sederhana (DIY)</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3000000</v>
+        <v>1500000</v>
       </c>
       <c r="E3" s="9">
         <f>C3*D3</f>
@@ -899,7 +907,7 @@
         </is>
       </c>
       <c r="H3" s="9">
-        <f>SUMIF($A$2:$A$44,G3,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G3,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -911,14 +919,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lantai / keramik / acian</t>
+          <t>Tambah stop kontak &amp; instalasi listrik</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3500000</v>
+        <v>1200000</v>
       </c>
       <c r="E4" s="9">
         <f>C4*D4</f>
@@ -930,7 +938,7 @@
         </is>
       </c>
       <c r="H4" s="9">
-        <f>SUMIF($A$2:$A$44,G4,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G4,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -942,14 +950,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Instalasi listrik + naik daya 4.400 VA</t>
+          <t>Lampu LED hangat</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>4000000</v>
+        <v>600000</v>
       </c>
       <c r="E5" s="9">
         <f>C5*D5</f>
@@ -961,7 +969,7 @@
         </is>
       </c>
       <c r="H5" s="9">
-        <f>SUMIF($A$2:$A$44,G5,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G5,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -973,14 +981,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Plumbing, wastafel &amp; saluran</t>
+          <t>Counter bar sederhana (kayu/besi hollow)</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2000000</v>
+        <v>1200000</v>
       </c>
       <c r="E6" s="9">
         <f>C6*D6</f>
@@ -992,7 +1000,7 @@
         </is>
       </c>
       <c r="H6" s="9">
-        <f>SUMIF($A$2:$A$44,G6,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G6,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -1004,14 +1012,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Meja bar/counter custom</t>
+          <t>Wastafel &amp; plumbing kecil</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>4000000</v>
+        <v>500000</v>
       </c>
       <c r="E7" s="9">
         <f>C7*D7</f>
@@ -1023,26 +1031,26 @@
         </is>
       </c>
       <c r="H7" s="9">
-        <f>SUMIF($A$2:$A$44,G7,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G7,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B. Renovasi</t>
+          <t>C. Bar Kopi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lampu &amp; exhaust fan</t>
+          <t>Moka pot 6 cup</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1500000</v>
+        <v>350000</v>
       </c>
       <c r="E8" s="9">
         <f>C8*D8</f>
@@ -1054,7 +1062,7 @@
         </is>
       </c>
       <c r="H8" s="9">
-        <f>SUMIF($A$2:$A$44,G8,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G8,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -1066,14 +1074,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mesin espresso 1 group (entry-level)</t>
+          <t>Grinder kopi elektrik (burr)</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>9500000</v>
+        <v>1000000</v>
       </c>
       <c r="E9" s="9">
         <f>C9*D9</f>
@@ -1085,7 +1093,7 @@
         </is>
       </c>
       <c r="H9" s="9">
-        <f>SUMIF($A$2:$A$44,G9,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G9,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -1097,14 +1105,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Grinder espresso</t>
+          <t>Set cold brew (toples kaca + filter)</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>3500000</v>
+        <v>300000</v>
       </c>
       <c r="E10" s="9">
         <f>C10*D10</f>
@@ -1116,7 +1124,7 @@
         </is>
       </c>
       <c r="H10" s="9">
-        <f>SUMIF($A$2:$A$44,G10,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G10,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -1128,14 +1136,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Barista tools (tamper, pitcher, timbangan, knock box)</t>
+          <t>Set manual brew (V60, kettle, timbangan)</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="E11" s="9">
         <f>C11*D11</f>
@@ -1147,7 +1155,7 @@
         </is>
       </c>
       <c r="H11" s="9">
-        <f>SUMIF($A$2:$A$44,G11,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G11,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -1159,14 +1167,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Set manual brew (V60, kettle leher angsa, server)</t>
+          <t>Blender</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>700000</v>
+        <v>800000</v>
       </c>
       <c r="E12" s="9">
         <f>C12*D12</f>
@@ -1178,7 +1186,7 @@
         </is>
       </c>
       <c r="H12" s="9">
-        <f>SUMIF($A$2:$A$44,G12,$E$2:$E$44)</f>
+        <f>SUMIF($A$2:$A$40,G12,$E$2:$E$40)</f>
         <v/>
       </c>
     </row>
@@ -1190,14 +1198,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Blender komersial</t>
+          <t>Water boiler 10 L</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1300000</v>
+        <v>1000000</v>
       </c>
       <c r="E13" s="9">
         <f>C13*D13</f>
@@ -1207,19 +1215,19 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C. Bar Kopi</t>
+          <t>D. Dapur</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Water boiler 20 L</t>
+          <t>Kompor 2 tungku + selang &amp; regulator</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1500000</v>
+        <v>800000</v>
       </c>
       <c r="E14" s="9">
         <f>C14*D14</f>
@@ -1234,14 +1242,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kompor 2 tungku + 2 tabung 12 kg isi + regulator</t>
+          <t>Tabung LPG 12 kg + isi</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2800000</v>
+        <v>900000</v>
       </c>
       <c r="E15" s="9">
         <f>C15*D15</f>
@@ -1256,14 +1264,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Griddle / pemanggang roti bakar</t>
+          <t>Plat pemanggang roti bakar</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1800000</v>
+        <v>500000</v>
       </c>
       <c r="E16" s="9">
         <f>C16*D16</f>
@@ -1278,14 +1286,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wajan besar &amp; perlengkapan gorengan</t>
+          <t>Wajan &amp; alat gorengan</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>700000</v>
+        <v>400000</v>
       </c>
       <c r="E17" s="9">
         <f>C17*D17</f>
@@ -1300,14 +1308,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Rice cooker 10 L</t>
+          <t>Rice cooker 5 L</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>900000</v>
+        <v>450000</v>
       </c>
       <c r="E18" s="9">
         <f>C18*D18</f>
@@ -1329,7 +1337,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>4200000</v>
+        <v>3800000</v>
       </c>
       <c r="E19" s="9">
         <f>C19*D19</f>
@@ -1344,14 +1352,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Chest freezer 200 L</t>
+          <t>Cool box es batu</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>2900000</v>
+        <v>250000</v>
       </c>
       <c r="E20" s="9">
         <f>C20*D20</f>
@@ -1366,14 +1374,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Peralatan masak (panci, wajan, pisau, talenan)</t>
+          <t>Peralatan masak</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1500000</v>
+        <v>800000</v>
       </c>
       <c r="E21" s="9">
         <f>C21*D21</f>
@@ -1388,14 +1396,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Peralatan saji 60 set (mangkok, piring, gelas, sendok)</t>
+          <t>Peralatan saji 40 set</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1000000</v>
+        <v>700000</v>
       </c>
       <c r="E22" s="9">
         <f>C22*D22</f>
@@ -1410,14 +1418,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Meja makan</t>
+          <t>Meja</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="E23" s="9">
         <f>C23*D23</f>
@@ -1436,7 +1444,7 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>100000</v>
@@ -1454,14 +1462,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Meja bar + 6 stool</t>
+          <t>Meja bar dinding + 4 stool</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>1500000</v>
+        <v>800000</v>
       </c>
       <c r="E25" s="9">
         <f>C25*D25</f>
@@ -1476,14 +1484,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rak &amp; lemari penyimpanan</t>
+          <t>Rak penyimpanan</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>800000</v>
+        <v>300000</v>
       </c>
       <c r="E26" s="9">
         <f>C26*D26</f>
@@ -1498,14 +1506,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tablet POS</t>
+          <t>Printer struk thermal bluetooth (POS di HP)</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>2800000</v>
+        <v>400000</v>
       </c>
       <c r="E27" s="9">
         <f>C27*D27</f>
@@ -1520,14 +1528,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Printer struk thermal</t>
+          <t>CCTV WiFi 2 kamera</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>700000</v>
+        <v>350000</v>
       </c>
       <c r="E28" s="9">
         <f>C28*D28</f>
@@ -1542,14 +1550,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Laci uang (cash drawer)</t>
+          <t>Pemasangan internet / WiFi</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>500000</v>
+        <v>300000</v>
       </c>
       <c r="E29" s="9">
         <f>C29*D29</f>
@@ -1564,14 +1572,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CCTV 4 kamera + DVR + HDD</t>
+          <t>Speaker bluetooth</t>
         </is>
       </c>
       <c r="C30" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>3000000</v>
+        <v>300000</v>
       </c>
       <c r="E30" s="9">
         <f>C30*D30</f>
@@ -1586,14 +1594,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Router WiFi + instalasi internet</t>
+          <t>APAR 3 kg</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>800000</v>
+        <v>350000</v>
       </c>
       <c r="E31" s="9">
         <f>C31*D31</f>
@@ -1603,19 +1611,19 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>F. Sistem</t>
+          <t>G. Branding</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Speaker / sound system</t>
+          <t>Logo (Canva / freelancer murah)</t>
         </is>
       </c>
       <c r="C32" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>1000000</v>
+        <v>300000</v>
       </c>
       <c r="E32" s="9">
         <f>C32*D32</f>
@@ -1625,19 +1633,19 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>F. Sistem</t>
+          <t>G. Branding</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>APAR (alat pemadam) 3 kg</t>
+          <t>Papan nama / spanduk besar</t>
         </is>
       </c>
       <c r="C33" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="E33" s="9">
         <f>C33*D33</f>
@@ -1652,14 +1660,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Logo &amp; brand kit (freelancer)</t>
+          <t>Menu board cetak</t>
         </is>
       </c>
       <c r="C34" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1500000</v>
+        <v>300000</v>
       </c>
       <c r="E34" s="9">
         <f>C34*D34</f>
@@ -1674,14 +1682,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Neon box / papan nama</t>
+          <t>Apron 4 pcs</t>
         </is>
       </c>
       <c r="C35" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>3000000</v>
+        <v>300000</v>
       </c>
       <c r="E35" s="9">
         <f>C35*D35</f>
@@ -1696,14 +1704,14 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Menu board + menu cetak</t>
+          <t>Stiker logo cup</t>
         </is>
       </c>
       <c r="C36" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>800000</v>
+        <v>300000</v>
       </c>
       <c r="E36" s="9">
         <f>C36*D36</f>
@@ -1713,19 +1721,19 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>G. Branding</t>
+          <t>H. Legal</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Seragam kaos &amp; apron 6 set</t>
+          <t>Surat lingkungan, domisili &amp; administrasi</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>900000</v>
+        <v>500000</v>
       </c>
       <c r="E37" s="9">
         <f>C37*D37</f>
@@ -1735,19 +1743,19 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>G. Branding</t>
+          <t>I. Stok Awal</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Stiker cup, stempel, kemasan</t>
+          <t>Bahan baku, kemasan, sabun dll</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>800000</v>
+        <v>4000000</v>
       </c>
       <c r="E38" s="9">
         <f>C38*D38</f>
@@ -1757,19 +1765,19 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>H. Legal</t>
+          <t>J. Marketing</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Surat lingkungan &amp; domisili</t>
+          <t>Pra-launch &amp; grand opening</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>500000</v>
+        <v>2000000</v>
       </c>
       <c r="E39" s="9">
         <f>C39*D39</f>
@@ -1779,19 +1787,19 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>H. Legal</t>
+          <t>K. Cadangan</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Uji sanitasi / SLHS &amp; administrasi</t>
+          <t>Dana cadangan / modal kerja</t>
         </is>
       </c>
       <c r="C40" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>500000</v>
+        <v>8700000</v>
       </c>
       <c r="E40" s="9">
         <f>C40*D40</f>
@@ -1799,101 +1807,13 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>H. Legal</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Materai, cetak &amp; lain-lain</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="2" t="n">
-        <v>500000</v>
-      </c>
-      <c r="E41" s="9">
-        <f>C41*D41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>I. Stok Awal</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Bahan baku, kemasan, gas, sabun dll</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="2" t="n">
-        <v>7000000</v>
-      </c>
-      <c r="E42" s="9">
-        <f>C42*D42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>J. Marketing</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Pra-launch &amp; grand opening</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="2" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="E43" s="9">
-        <f>C43*D43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>K. Cadangan</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Dana cadangan / modal kerja</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="2" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="E44" s="9">
-        <f>C44*D44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>TOTAL INVESTASI AWAL</t>
         </is>
       </c>
-      <c r="E45" s="6">
-        <f>SUM(E2:E44)</f>
+      <c r="E41" s="6">
+        <f>SUM(E2:E40)</f>
         <v/>
       </c>
     </row>
@@ -1908,7 +1828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2006,7 +1926,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Es kopi susu gula aren (espresso)</t>
+          <t>Kopi Susu Warkop (cold brew + SKM)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2015,10 +1935,10 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>7500</v>
+        <v>4500</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>18000</v>
+        <v>10000</v>
       </c>
       <c r="E4" s="10">
         <f>C4/D4</f>
@@ -2032,7 +1952,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kopi susu warkop signature (espresso + SKM)</t>
+          <t>Es Kopi Susu Gula Aren (cold brew)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2041,7 +1961,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>13000</v>
@@ -2058,7 +1978,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Americano / long black</t>
+          <t>Kopi seduh V60 beans lokal</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2067,10 +1987,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3800</v>
+        <v>3500</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13000</v>
+        <v>12000</v>
       </c>
       <c r="E6" s="10">
         <f>C6/D6</f>
@@ -2084,7 +2004,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Manual brew V60 (beans lokal)</t>
+          <t>Es teh manis jumbo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2093,10 +2013,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>6000</v>
+        <v>2000</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="E7" s="10">
         <f>C7/D7</f>
@@ -2110,7 +2030,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Es teh manis jumbo</t>
+          <t>Es jeruk</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2119,10 +2039,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2000</v>
+        <v>3500</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="E8" s="10">
         <f>C8/D8</f>
@@ -2136,7 +2056,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Es jeruk / jeruk peras</t>
+          <t>Susu jahe / wedang jahe</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2145,7 +2065,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>8000</v>
@@ -2162,16 +2082,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Susu jahe / wedang jahe</t>
+          <t>Indomie rebus/goreng polos</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Minuman</t>
+          <t>Makanan</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>8000</v>
@@ -2188,7 +2108,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Indomie rebus/goreng polos</t>
+          <t>Indomie + telur</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2197,10 +2117,10 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>4500</v>
+        <v>6900</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="E11" s="10">
         <f>C11/D11</f>
@@ -2214,7 +2134,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Indomie + telur</t>
+          <t>Indomie Special (telur, kornet, keju)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2223,10 +2143,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>6900</v>
+        <v>9500</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="E12" s="10">
         <f>C12/D12</f>
@@ -2240,7 +2160,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Indomie special (telur, kornet, keju)</t>
+          <t>Mie nyemek level pedas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2249,10 +2169,10 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>10500</v>
+        <v>7000</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>20000</v>
+        <v>14000</v>
       </c>
       <c r="E13" s="10">
         <f>C13/D13</f>
@@ -2266,7 +2186,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mie nyemek level pedas</t>
+          <t>Nasi telor + sambal + kerupuk</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2275,10 +2195,10 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>7500</v>
+        <v>4500</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E14" s="10">
         <f>C14/D14</f>
@@ -2292,7 +2212,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Nasi telor + sambal + kerupuk</t>
+          <t>Nasi goreng warkop</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2301,10 +2221,10 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>4500</v>
+        <v>7000</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E15" s="10">
         <f>C15/D15</f>
@@ -2318,7 +2238,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nasi goreng warkop</t>
+          <t>Roti bakar coklat keju</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2327,10 +2247,10 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>7500</v>
+        <v>5500</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>16000</v>
+        <v>13000</v>
       </c>
       <c r="E16" s="10">
         <f>C16/D16</f>
@@ -2344,7 +2264,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Rice bowl ayam sambal matah</t>
+          <t>Pisang bakar coklat</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2353,10 +2273,10 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>9000</v>
+        <v>4500</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="E17" s="10">
         <f>C17/D17</f>
@@ -2370,19 +2290,19 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Roti bakar coklat keju</t>
+          <t>Gorengan titip jual (per biji)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Makanan</t>
+          <t>Camilan</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>6100</v>
+        <v>1400</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E18" s="10">
         <f>C18/D18</f>
@@ -2390,84 +2310,6 @@
       </c>
       <c r="F18" s="9">
         <f>D18-C18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Pisang bakar / pisang keju</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Makanan</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D19" s="2" t="n">
-        <v>12000</v>
-      </c>
-      <c r="E19" s="10">
-        <f>C19/D19</f>
-        <v/>
-      </c>
-      <c r="F19" s="9">
-        <f>D19-C19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Gorengan (per biji)</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Camilan</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D20" s="2" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E20" s="10">
-        <f>C20/D20</f>
-        <v/>
-      </c>
-      <c r="F20" s="9">
-        <f>D20-C20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Kentang goreng</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Camilan</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>5500</v>
-      </c>
-      <c r="D21" s="2" t="n">
-        <v>13000</v>
-      </c>
-      <c r="E21" s="10">
-        <f>C21/D21</f>
-        <v/>
-      </c>
-      <c r="F21" s="9">
-        <f>D21-C21</f>
         <v/>
       </c>
     </row>
@@ -2592,11 +2434,11 @@
         <v/>
       </c>
       <c r="J2" s="9">
-        <f>I2+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I2+Asumsi!$B$22+IF(A2&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K2" s="9">
-        <f>-Modal!$E$45+J2</f>
+        <f>-Modal!$E$41+J2</f>
         <v/>
       </c>
     </row>
@@ -2637,7 +2479,7 @@
         <v/>
       </c>
       <c r="J3" s="9">
-        <f>I3+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I3+Asumsi!$B$22+IF(A3&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K3" s="9">
@@ -2682,7 +2524,7 @@
         <v/>
       </c>
       <c r="J4" s="9">
-        <f>I4+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I4+Asumsi!$B$22+IF(A4&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K4" s="9">
@@ -2727,7 +2569,7 @@
         <v/>
       </c>
       <c r="J5" s="9">
-        <f>I5+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I5+Asumsi!$B$22+IF(A5&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K5" s="9">
@@ -2772,7 +2614,7 @@
         <v/>
       </c>
       <c r="J6" s="9">
-        <f>I6+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I6+Asumsi!$B$22+IF(A6&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K6" s="9">
@@ -2817,7 +2659,7 @@
         <v/>
       </c>
       <c r="J7" s="9">
-        <f>I7+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I7+Asumsi!$B$22+IF(A7&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K7" s="9">
@@ -2862,7 +2704,7 @@
         <v/>
       </c>
       <c r="J8" s="9">
-        <f>I8+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I8+Asumsi!$B$22+IF(A8&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K8" s="9">
@@ -2907,7 +2749,7 @@
         <v/>
       </c>
       <c r="J9" s="9">
-        <f>I9+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I9+Asumsi!$B$22+IF(A9&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K9" s="9">
@@ -2952,7 +2794,7 @@
         <v/>
       </c>
       <c r="J10" s="9">
-        <f>I10+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I10+Asumsi!$B$22+IF(A10&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K10" s="9">
@@ -2997,7 +2839,7 @@
         <v/>
       </c>
       <c r="J11" s="9">
-        <f>I11+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I11+Asumsi!$B$22+IF(A11&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K11" s="9">
@@ -3042,7 +2884,7 @@
         <v/>
       </c>
       <c r="J12" s="9">
-        <f>I12+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I12+Asumsi!$B$22+IF(A12&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K12" s="9">
@@ -3087,7 +2929,7 @@
         <v/>
       </c>
       <c r="J13" s="9">
-        <f>I13+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>I13+Asumsi!$B$22+IF(A13&lt;=Asumsi!$D$25,Asumsi!$B$12,0)</f>
         <v/>
       </c>
       <c r="K13" s="9">
@@ -3137,7 +2979,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>* Arus kas = laba bersih + penyusutan + sewa (sewa tahun-1 sudah dibayar di muka dalam modal). Mulai tahun ke-2, sisihkan sewa tiap bulan.</t>
+          <t>* Arus kas = laba bersih + penyusutan (+ sewa pada bulan yang sudah dibayar di muka dalam modal). Sisihkan Rp1,2jt/bulan sejak bulan 1 untuk membayar sewa periode berikutnya.</t>
         </is>
       </c>
     </row>
@@ -3197,13 +3039,13 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>180</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -3213,13 +3055,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>19000</v>
+        <v>16000</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>20000</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="4">
@@ -3362,15 +3204,15 @@
         </is>
       </c>
       <c r="B11" s="9">
-        <f>B9+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>B9+Asumsi!$B$22</f>
         <v/>
       </c>
       <c r="C11" s="9">
-        <f>C9+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>C9+Asumsi!$B$22</f>
         <v/>
       </c>
       <c r="D11" s="9">
-        <f>D9+Asumsi!$B$22+Asumsi!$B$12</f>
+        <f>D9+Asumsi!$B$22</f>
         <v/>
       </c>
     </row>
@@ -3381,15 +3223,15 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>Modal!$E$45/B11</f>
+        <f>Modal!$E$41/B11</f>
         <v/>
       </c>
       <c r="C12" s="11">
-        <f>Modal!$E$45/C11</f>
+        <f>Modal!$E$41/C11</f>
         <v/>
       </c>
       <c r="D12" s="11">
-        <f>Modal!$E$45/D11</f>
+        <f>Modal!$E$41/D11</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Ubah masterplan ke menu warkop Kuningan autentik
Naik kelas difokuskan pada tempat (bersih, rapi, nyaman untuk Gen Z),
bukan menu kafe. Menu, alat, SOP kebersihan, roadmap upgrade, model
keuangan, dan PDF diperbarui (BEP ±47 transaksi/hari).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjJU715WJBpBotxgoH1Pwh
</commit_message>
<xml_diff>
--- a/warkop/Model-Keuangan-Warkop.xlsx
+++ b/warkop/Model-Keuangan-Warkop.xlsx
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>16000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="4">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.42</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="5">
@@ -640,11 +640,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Penyusutan alat (± Rp20,4jt / 48 bln)</t>
+          <t>Penyusutan alat (± Rp19,4jt / 48 bln)</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>450000</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="23">
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30">
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31">
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32">
@@ -740,7 +740,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="33">
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34">
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="36">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="37">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -804,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="H2" s="9">
-        <f>SUMIF($A$2:$A$40,G2,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G2,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="H3" s="9">
-        <f>SUMIF($A$2:$A$40,G3,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G3,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
@@ -934,11 +934,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>C. Bar Kopi</t>
+          <t>C. Bar Minuman</t>
         </is>
       </c>
       <c r="H4" s="9">
-        <f>SUMIF($A$2:$A$40,G4,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G4,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="H5" s="9">
-        <f>SUMIF($A$2:$A$40,G5,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G5,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="H6" s="9">
-        <f>SUMIF($A$2:$A$40,G6,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G6,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
@@ -1031,26 +1031,26 @@
         </is>
       </c>
       <c r="H7" s="9">
-        <f>SUMIF($A$2:$A$40,G7,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G7,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C. Bar Kopi</t>
+          <t>C. Bar Minuman</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Moka pot 6 cup</t>
+          <t>Rak &amp; gantungan renteng sachet</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>350000</v>
+        <v>300000</v>
       </c>
       <c r="E8" s="9">
         <f>C8*D8</f>
@@ -1062,19 +1062,19 @@
         </is>
       </c>
       <c r="H8" s="9">
-        <f>SUMIF($A$2:$A$40,G8,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G8,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C. Bar Kopi</t>
+          <t>C. Bar Minuman</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Grinder kopi elektrik (burr)</t>
+          <t>Water boiler 10 L</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
@@ -1093,26 +1093,26 @@
         </is>
       </c>
       <c r="H9" s="9">
-        <f>SUMIF($A$2:$A$40,G9,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G9,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C. Bar Kopi</t>
+          <t>C. Bar Minuman</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Set cold brew (toples kaca + filter)</t>
+          <t>Blender (es sachet/Pop Ice)</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>300000</v>
+        <v>800000</v>
       </c>
       <c r="E10" s="9">
         <f>C10*D10</f>
@@ -1124,26 +1124,26 @@
         </is>
       </c>
       <c r="H10" s="9">
-        <f>SUMIF($A$2:$A$40,G10,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G10,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C. Bar Kopi</t>
+          <t>C. Bar Minuman</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Set manual brew (V60, kettle, timbangan)</t>
+          <t>Panci besar burjo &amp; ketan hitam</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="E11" s="9">
         <f>C11*D11</f>
@@ -1155,26 +1155,26 @@
         </is>
       </c>
       <c r="H11" s="9">
-        <f>SUMIF($A$2:$A$40,G11,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G11,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C. Bar Kopi</t>
+          <t>C. Bar Minuman</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Blender</t>
+          <t>Teko, gelas takar &amp; termos</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>800000</v>
+        <v>200000</v>
       </c>
       <c r="E12" s="9">
         <f>C12*D12</f>
@@ -1186,26 +1186,26 @@
         </is>
       </c>
       <c r="H12" s="9">
-        <f>SUMIF($A$2:$A$40,G12,$E$2:$E$40)</f>
+        <f>SUMIF($A$2:$A$41,G12,$E$2:$E$41)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C. Bar Kopi</t>
+          <t>D. Dapur</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Water boiler 10 L</t>
+          <t>Kompor 2 tungku + selang &amp; regulator</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1000000</v>
+        <v>800000</v>
       </c>
       <c r="E13" s="9">
         <f>C13*D13</f>
@@ -1220,14 +1220,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kompor 2 tungku + selang &amp; regulator</t>
+          <t>Tabung LPG 12 kg + isi</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>800000</v>
+        <v>900000</v>
       </c>
       <c r="E14" s="9">
         <f>C14*D14</f>
@@ -1242,14 +1242,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tabung LPG 12 kg + isi</t>
+          <t>Plat pemanggang roti bakar</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>900000</v>
+        <v>500000</v>
       </c>
       <c r="E15" s="9">
         <f>C15*D15</f>
@@ -1264,14 +1264,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Plat pemanggang roti bakar</t>
+          <t>Wajan &amp; alat gorengan</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="E16" s="9">
         <f>C16*D16</f>
@@ -1286,14 +1286,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wajan &amp; alat gorengan</t>
+          <t>Rice cooker 5 L</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>400000</v>
+        <v>450000</v>
       </c>
       <c r="E17" s="9">
         <f>C17*D17</f>
@@ -1308,14 +1308,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Rice cooker 5 L</t>
+          <t>Kulkas showcase 1 pintu</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>450000</v>
+        <v>3800000</v>
       </c>
       <c r="E18" s="9">
         <f>C18*D18</f>
@@ -1330,14 +1330,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kulkas showcase 1 pintu</t>
+          <t>Cool box es batu</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>3800000</v>
+        <v>250000</v>
       </c>
       <c r="E19" s="9">
         <f>C19*D19</f>
@@ -1352,14 +1352,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cool box es batu</t>
+          <t>Peralatan masak</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>250000</v>
+        <v>800000</v>
       </c>
       <c r="E20" s="9">
         <f>C20*D20</f>
@@ -1374,14 +1374,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Peralatan masak</t>
+          <t>Peralatan saji 40 set</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>800000</v>
+        <v>700000</v>
       </c>
       <c r="E21" s="9">
         <f>C21*D21</f>
@@ -1391,19 +1391,19 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>D. Dapur</t>
+          <t>E. Furniture</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Peralatan saji 40 set</t>
+          <t>Meja</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>700000</v>
+        <v>400000</v>
       </c>
       <c r="E22" s="9">
         <f>C22*D22</f>
@@ -1418,14 +1418,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Meja</t>
+          <t>Kursi / bangku</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>400000</v>
+        <v>100000</v>
       </c>
       <c r="E23" s="9">
         <f>C23*D23</f>
@@ -1440,14 +1440,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kursi / bangku</t>
+          <t>Meja bar dinding + 4 stool</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>100000</v>
+        <v>800000</v>
       </c>
       <c r="E24" s="9">
         <f>C24*D24</f>
@@ -1462,14 +1462,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Meja bar dinding + 4 stool</t>
+          <t>Rak penyimpanan</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>800000</v>
+        <v>300000</v>
       </c>
       <c r="E25" s="9">
         <f>C25*D25</f>
@@ -1484,11 +1484,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rak penyimpanan</t>
+          <t>Kipas angin dinding</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>300000</v>
@@ -1660,14 +1660,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Menu board cetak</t>
+          <t>Neon flex tulisan (spot foto)</t>
         </is>
       </c>
       <c r="C34" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>300000</v>
+        <v>500000</v>
       </c>
       <c r="E34" s="9">
         <f>C34*D34</f>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Apron 4 pcs</t>
+          <t>Menu board berfoto</t>
         </is>
       </c>
       <c r="C35" s="7" t="n">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Stiker logo cup</t>
+          <t>Kaos seragam &amp; apron 4 set</t>
         </is>
       </c>
       <c r="C36" s="7" t="n">
@@ -1721,19 +1721,19 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>H. Legal</t>
+          <t>G. Branding</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Surat lingkungan, domisili &amp; administrasi</t>
+          <t>Stiker logo cup</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>500000</v>
+        <v>300000</v>
       </c>
       <c r="E37" s="9">
         <f>C37*D37</f>
@@ -1743,19 +1743,19 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>I. Stok Awal</t>
+          <t>H. Legal</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bahan baku, kemasan, sabun dll</t>
+          <t>Surat lingkungan, domisili &amp; administrasi</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>4000000</v>
+        <v>500000</v>
       </c>
       <c r="E38" s="9">
         <f>C38*D38</f>
@@ -1765,19 +1765,19 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>J. Marketing</t>
+          <t>I. Stok Awal</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Pra-launch &amp; grand opening</t>
+          <t>Bahan baku, kemasan, sabun dll</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>2000000</v>
+        <v>4000000</v>
       </c>
       <c r="E39" s="9">
         <f>C39*D39</f>
@@ -1787,19 +1787,19 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>K. Cadangan</t>
+          <t>J. Marketing</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Dana cadangan / modal kerja</t>
+          <t>Pra-launch &amp; grand opening</t>
         </is>
       </c>
       <c r="C40" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>8700000</v>
+        <v>2000000</v>
       </c>
       <c r="E40" s="9">
         <f>C40*D40</f>
@@ -1807,13 +1807,35 @@
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="5" t="inlineStr">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>K. Cadangan</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Dana cadangan / modal kerja</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>9200000</v>
+      </c>
+      <c r="E41" s="9">
+        <f>C41*D41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>TOTAL INVESTASI AWAL</t>
         </is>
       </c>
-      <c r="E41" s="6">
-        <f>SUM(E2:E40)</f>
+      <c r="E42" s="6">
+        <f>SUM(E2:E41)</f>
         <v/>
       </c>
     </row>
@@ -1828,7 +1850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1874,7 +1896,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kopi hitam sachet / tubruk</t>
+          <t>Kopi sachet panas (Kapal Api, ABC, Torabika, Good Day, Luwak)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1883,10 +1905,10 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2300</v>
+        <v>1800</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="E2" s="10">
         <f>C2/D2</f>
@@ -1900,7 +1922,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kopi susu sachet (panas/es)</t>
+          <t>Kopi sachet es</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1909,10 +1931,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>2800</v>
+        <v>2300</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="E3" s="10">
         <f>C3/D3</f>
@@ -1926,7 +1948,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kopi Susu Warkop (cold brew + SKM)</t>
+          <t>Kopi hitam tubruk</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1935,10 +1957,10 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>4500</v>
+        <v>1200</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="E4" s="10">
         <f>C4/D4</f>
@@ -1952,7 +1974,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Es Kopi Susu Gula Aren (cold brew)</t>
+          <t>Teh manis panas</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1961,10 +1983,10 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>6000</v>
+        <v>800</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13000</v>
+        <v>3000</v>
       </c>
       <c r="E5" s="10">
         <f>C5/D5</f>
@@ -1978,7 +2000,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kopi seduh V60 beans lokal</t>
+          <t>Es teh manis jumbo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1987,10 +2009,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3500</v>
+        <v>1500</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>12000</v>
+        <v>5000</v>
       </c>
       <c r="E6" s="10">
         <f>C6/D6</f>
@@ -2004,7 +2026,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Es teh manis jumbo</t>
+          <t>Susu jahe / jahe sachet</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2030,7 +2052,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Es jeruk</t>
+          <t>Susu putih / cokelat (SKM)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2039,10 +2061,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>8000</v>
+        <v>5000</v>
       </c>
       <c r="E8" s="10">
         <f>C8/D8</f>
@@ -2056,7 +2078,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Susu jahe / wedang jahe</t>
+          <t>Extra Joss / Kuku Bima susu</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2068,7 +2090,7 @@
         <v>3000</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>8000</v>
+        <v>6000</v>
       </c>
       <c r="E9" s="10">
         <f>C9/D9</f>
@@ -2082,19 +2104,19 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Indomie rebus/goreng polos</t>
+          <t>Minuman sachet es (Nutrisari, Milo, Pop Ice)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Makanan</t>
+          <t>Minuman</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>4500</v>
+        <v>2300</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>8000</v>
+        <v>5000</v>
       </c>
       <c r="E10" s="10">
         <f>C10/D10</f>
@@ -2108,7 +2130,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Indomie + telur</t>
+          <t>Indomie rebus/goreng (semua varian)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2117,10 +2139,10 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>6900</v>
+        <v>4200</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>12000</v>
+        <v>8000</v>
       </c>
       <c r="E11" s="10">
         <f>C11/D11</f>
@@ -2134,7 +2156,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Indomie Special (telur, kornet, keju)</t>
+          <t>Indomie telor</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2143,10 +2165,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>9500</v>
+        <v>6500</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>18000</v>
+        <v>12000</v>
       </c>
       <c r="E12" s="10">
         <f>C12/D12</f>
@@ -2160,7 +2182,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mie nyemek level pedas</t>
+          <t>Indomie telor kornet</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2169,10 +2191,10 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>14000</v>
+        <v>15000</v>
       </c>
       <c r="E13" s="10">
         <f>C13/D13</f>
@@ -2186,7 +2208,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Nasi telor + sambal + kerupuk</t>
+          <t>Indomie double telor</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2195,10 +2217,10 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>4500</v>
+        <v>10200</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>10000</v>
+        <v>18000</v>
       </c>
       <c r="E14" s="10">
         <f>C14/D14</f>
@@ -2212,7 +2234,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Nasi goreng warkop</t>
+          <t>Indomie nyemek pedas</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2221,10 +2243,10 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>7000</v>
+        <v>6800</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
       <c r="E15" s="10">
         <f>C15/D15</f>
@@ -2238,7 +2260,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Roti bakar coklat keju</t>
+          <t>Burjo (bubur kacang ijo)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2247,10 +2269,10 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5500</v>
+        <v>2500</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13000</v>
+        <v>7000</v>
       </c>
       <c r="E16" s="10">
         <f>C16/D16</f>
@@ -2264,7 +2286,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pisang bakar coklat</t>
+          <t>Burjo ketan hitam</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2273,10 +2295,10 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="E17" s="10">
         <f>C17/D17</f>
@@ -2290,19 +2312,19 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Gorengan titip jual (per biji)</t>
+          <t>Nasi telor + kerupuk</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Camilan</t>
+          <t>Makanan</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1400</v>
+        <v>4500</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="E18" s="10">
         <f>C18/D18</f>
@@ -2310,6 +2332,110 @@
       </c>
       <c r="F18" s="9">
         <f>D18-C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Nasi goreng telor</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Makanan</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>13000</v>
+      </c>
+      <c r="E19" s="10">
+        <f>C19/D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="9">
+        <f>D19-C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Magelangan (nasi goreng campur mie)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Makanan</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>7000</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E20" s="10">
+        <f>C20/D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="9">
+        <f>D20-C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Roti bakar (cokelat/keju/srikaya)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Makanan</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E21" s="10">
+        <f>C21/D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="9">
+        <f>D21-C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Gorengan titip jual (per biji)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Camilan</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E22" s="10">
+        <f>C22/D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="9">
+        <f>D22-C22</f>
         <v/>
       </c>
     </row>
@@ -2438,7 +2564,7 @@
         <v/>
       </c>
       <c r="K2" s="9">
-        <f>-Modal!$E$41+J2</f>
+        <f>-Modal!$E$42+J2</f>
         <v/>
       </c>
     </row>
@@ -3039,13 +3165,13 @@
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3">
@@ -3055,13 +3181,13 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>14000</v>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>15000</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="D3" s="2" t="n">
         <v>16000</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>17000</v>
       </c>
     </row>
     <row r="4">
@@ -3223,15 +3349,15 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>Modal!$E$41/B11</f>
+        <f>Modal!$E$42/B11</f>
         <v/>
       </c>
       <c r="C12" s="11">
-        <f>Modal!$E$41/C11</f>
+        <f>Modal!$E$42/C11</f>
         <v/>
       </c>
       <c r="D12" s="11">
-        <f>Modal!$E$41/D11</f>
+        <f>Modal!$E$42/D11</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Sesuaikan masterplan dengan sewa ruko Rp 2,5 juta/bulan
Sewa 6 bulan Rp 15 juta, alokasi modal Rp 50 juta disusun ulang,
biaya tetap Rp 12,5 juta/bulan, BEP ±52 transaksi/hari. Excel dan
PDF ikut diperbarui.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NjJU715WJBpBotxgoH1Pwh
</commit_message>
<xml_diff>
--- a/warkop/Model-Keuangan-Warkop.xlsx
+++ b/warkop/Model-Keuangan-Warkop.xlsx
@@ -540,11 +540,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sewa (Rp1,2jt/bulan)</t>
+          <t>Sewa ruko (Rp2,5jt/bulan)</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>1200000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="13">
@@ -640,7 +640,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Penyusutan alat (± Rp19,4jt / 48 bln)</t>
+          <t>Penyusutan alat (± Rp18,4jt / 48 bln)</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -857,14 +857,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sewa kios 3x8 m + teras, 6 bulan di muka (Rp1,2jt/bln)</t>
+          <t>Sewa ruko 1 lantai ± 4x10 m, 6 bulan di muka (Rp2,5jt/bln)</t>
         </is>
       </c>
       <c r="C2" s="7" t="n">
         <v>6</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1200000</v>
+        <v>2500000</v>
       </c>
       <c r="E2" s="9">
         <f>C2*D2</f>
@@ -888,14 +888,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cat &amp; mural sederhana (DIY)</t>
+          <t>Cat &amp; finishing (DIY)</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1500000</v>
+        <v>1300000</v>
       </c>
       <c r="E3" s="9">
         <f>C3*D3</f>
@@ -926,7 +926,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1200000</v>
+        <v>900000</v>
       </c>
       <c r="E4" s="9">
         <f>C4*D4</f>
@@ -988,7 +988,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1200000</v>
+        <v>1000000</v>
       </c>
       <c r="E6" s="9">
         <f>C6*D6</f>
@@ -1012,14 +1012,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wastafel &amp; plumbing kecil</t>
+          <t>Wastafel &amp; perbaikan kecil</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>500000</v>
+        <v>200000</v>
       </c>
       <c r="E7" s="9">
         <f>C7*D7</f>
@@ -1308,14 +1308,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Kulkas showcase 1 pintu</t>
+          <t>Kulkas showcase 1 pintu (bekas kondisi baik)</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>3800000</v>
+        <v>2800000</v>
       </c>
       <c r="E18" s="9">
         <f>C18*D18</f>
@@ -1638,14 +1638,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Papan nama / spanduk besar</t>
+          <t>Spanduk papan nama (papan permanen menyusul)</t>
         </is>
       </c>
       <c r="C33" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="E33" s="9">
         <f>C33*D33</f>
@@ -1777,7 +1777,7 @@
         <v>1</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>4000000</v>
+        <v>3000000</v>
       </c>
       <c r="E39" s="9">
         <f>C39*D39</f>
@@ -1799,7 +1799,7 @@
         <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>2000000</v>
+        <v>1500000</v>
       </c>
       <c r="E40" s="9">
         <f>C40*D40</f>
@@ -1821,7 +1821,7 @@
         <v>1</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>9200000</v>
+        <v>5400000</v>
       </c>
       <c r="E41" s="9">
         <f>C41*D41</f>
@@ -3105,7 +3105,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>* Arus kas = laba bersih + penyusutan (+ sewa pada bulan yang sudah dibayar di muka dalam modal). Sisihkan Rp1,2jt/bulan sejak bulan 1 untuk membayar sewa periode berikutnya.</t>
+          <t>* Arus kas = laba bersih + penyusutan (+ sewa pada bulan yang sudah dibayar di muka dalam modal). Sisihkan Rp2,5jt/bulan sejak bulan 1 untuk membayar sewa periode berikutnya.</t>
         </is>
       </c>
     </row>

</xml_diff>